<commit_message>
Make sample calibration error bars visible
</commit_message>
<xml_diff>
--- a/samples/sample_03_abs_error.xlsx
+++ b/samples/sample_03_abs_error.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sample" sheetId="1" r:id="Rb5f4c641daf346ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sample" sheetId="1" r:id="Re7faf0ba2f7c4a53"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -296,7 +296,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="5" t="str">
-        <x:v>练习：预设会启用 absorbance_sd 作为 Y 误差棒，并叠加一次线性拟合。</x:v>
+        <x:v>练习：预设会启用清晰可见的 absorbance_sd 作为 Y 误差棒，并叠加一次线性拟合。</x:v>
       </x:c>
       <x:c r="B3" s="5" t="str"/>
       <x:c r="C3" s="5" t="str"/>
@@ -306,7 +306,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="5" t="str">
-        <x:v>进阶：查看中点参考线、误差棒和拟合指标是否支持实验判断。</x:v>
+        <x:v>进阶：误差棒由两次重复测量的示例标准差给出，可检查中点参考线和拟合指标。</x:v>
       </x:c>
       <x:c r="B4" s="5" t="str"/>
       <x:c r="C4" s="5" t="str"/>
@@ -382,10 +382,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B10" s="15" t="n">
-        <x:v>0.006</x:v>
+        <x:v>0.0008</x:v>
       </x:c>
       <x:c r="C10" s="15" t="n">
-        <x:v>0.004</x:v>
+        <x:v>0.0092</x:v>
       </x:c>
       <x:c r="D10" s="15" t="n">
         <x:v>0.005</x:v>
@@ -397,7 +397,7 @@
         <x:v>-0.001</x:v>
       </x:c>
       <x:c r="G10" t="n">
-        <x:v>0.0014</x:v>
+        <x:v>0.006</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -405,10 +405,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B11" s="15" t="n">
-        <x:v>0.117</x:v>
+        <x:v>0.1087</x:v>
       </x:c>
       <x:c r="C11" s="15" t="n">
-        <x:v>0.123</x:v>
+        <x:v>0.1313</x:v>
       </x:c>
       <x:c r="D11" s="15" t="n">
         <x:v>0.12</x:v>
@@ -420,7 +420,7 @@
         <x:v>-0.007</x:v>
       </x:c>
       <x:c r="G11" t="n">
-        <x:v>0.0042</x:v>
+        <x:v>0.016</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -428,10 +428,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B12" s="15" t="n">
-        <x:v>0.238</x:v>
+        <x:v>0.2283</x:v>
       </x:c>
       <x:c r="C12" s="15" t="n">
-        <x:v>0.244</x:v>
+        <x:v>0.2537</x:v>
       </x:c>
       <x:c r="D12" s="15" t="n">
         <x:v>0.241</x:v>
@@ -443,7 +443,7 @@
         <x:v>-0.007</x:v>
       </x:c>
       <x:c r="G12" t="n">
-        <x:v>0.0042</x:v>
+        <x:v>0.018</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -451,10 +451,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B13" s="15" t="n">
-        <x:v>0.362</x:v>
+        <x:v>0.3449</x:v>
       </x:c>
       <x:c r="C13" s="15" t="n">
-        <x:v>0.356</x:v>
+        <x:v>0.3731</x:v>
       </x:c>
       <x:c r="D13" s="15" t="n">
         <x:v>0.359</x:v>
@@ -466,7 +466,7 @@
         <x:v>-0.01</x:v>
       </x:c>
       <x:c r="G13" t="n">
-        <x:v>0.0042</x:v>
+        <x:v>0.02</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -474,10 +474,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B14" s="15" t="n">
-        <x:v>0.475</x:v>
+        <x:v>0.4635</x:v>
       </x:c>
       <x:c r="C14" s="15" t="n">
-        <x:v>0.486</x:v>
+        <x:v>0.4975</x:v>
       </x:c>
       <x:c r="D14" s="15" t="n">
         <x:v>0.4805</x:v>
@@ -489,7 +489,7 @@
         <x:v>-0.0095</x:v>
       </x:c>
       <x:c r="G14" t="n">
-        <x:v>0.0078</x:v>
+        <x:v>0.024</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -497,10 +497,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B15" s="15" t="n">
-        <x:v>0.602</x:v>
+        <x:v>0.5806</x:v>
       </x:c>
       <x:c r="C15" s="15" t="n">
-        <x:v>0.596</x:v>
+        <x:v>0.6174</x:v>
       </x:c>
       <x:c r="D15" s="15" t="n">
         <x:v>0.599</x:v>
@@ -512,7 +512,7 @@
         <x:v>-0.012</x:v>
       </x:c>
       <x:c r="G15" t="n">
-        <x:v>0.0042</x:v>
+        <x:v>0.026</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -520,10 +520,10 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B16" s="15" t="n">
-        <x:v>0.724</x:v>
+        <x:v>0.7063</x:v>
       </x:c>
       <x:c r="C16" s="15" t="n">
-        <x:v>0.731</x:v>
+        <x:v>0.7487</x:v>
       </x:c>
       <x:c r="D16" s="15" t="n">
         <x:v>0.7275</x:v>
@@ -535,7 +535,7 @@
         <x:v>-0.0045</x:v>
       </x:c>
       <x:c r="G16" t="n">
-        <x:v>0.0049</x:v>
+        <x:v>0.03</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -543,10 +543,10 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B17" s="15" t="n">
-        <x:v>0.851</x:v>
+        <x:v>0.8244</x:v>
       </x:c>
       <x:c r="C17" s="15" t="n">
-        <x:v>0.843</x:v>
+        <x:v>0.8696</x:v>
       </x:c>
       <x:c r="D17" s="15" t="n">
         <x:v>0.847</x:v>
@@ -558,7 +558,7 @@
         <x:v>-0.006</x:v>
       </x:c>
       <x:c r="G17" t="n">
-        <x:v>0.0057</x:v>
+        <x:v>0.032</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -566,10 +566,10 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B18" s="15" t="n">
-        <x:v>0.958</x:v>
+        <x:v>0.939</x:v>
       </x:c>
       <x:c r="C18" s="15" t="n">
-        <x:v>0.971</x:v>
+        <x:v>0.99</x:v>
       </x:c>
       <x:c r="D18" s="15" t="n">
         <x:v>0.9645</x:v>
@@ -581,7 +581,7 @@
         <x:v>-0.0095</x:v>
       </x:c>
       <x:c r="G18" t="n">
-        <x:v>0.0092</x:v>
+        <x:v>0.036</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -589,10 +589,10 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B19" s="15" t="n">
-        <x:v>1.082</x:v>
+        <x:v>1.0602</x:v>
       </x:c>
       <x:c r="C19" s="15" t="n">
-        <x:v>1.095</x:v>
+        <x:v>1.1168</x:v>
       </x:c>
       <x:c r="D19" s="15" t="n">
         <x:v>1.0885</x:v>
@@ -604,7 +604,7 @@
         <x:v>-0.0065</x:v>
       </x:c>
       <x:c r="G19" t="n">
-        <x:v>0.0092</x:v>
+        <x:v>0.04</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -612,10 +612,10 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="B20" s="15" t="n">
-        <x:v>1.214</x:v>
+        <x:v>1.1774</x:v>
       </x:c>
       <x:c r="C20" s="15" t="n">
-        <x:v>1.203</x:v>
+        <x:v>1.2396</x:v>
       </x:c>
       <x:c r="D20" s="15" t="n">
         <x:v>1.2085</x:v>
@@ -627,7 +627,7 @@
         <x:v>-0.0075</x:v>
       </x:c>
       <x:c r="G20" t="n">
-        <x:v>0.0078</x:v>
+        <x:v>0.044</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>